<commit_message>
update affiliate product links
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -1,49 +1,152 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="390" yWindow="615" windowWidth="13095" windowHeight="7620"/>
   </bookViews>
   <sheets>
-    <sheet name="Affiliate Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Affiliate Products" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Shopee URL</t>
+  </si>
+  <si>
+    <t>Lazada URL</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>ตัวอย่างสินค้า 1</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>ตัวอย่างสินค้า 2</t>
+  </si>
+  <si>
+    <t>ตัวอย่างสินค้า 3</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/Lk7rJ9Beg</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/AUqtyHxaLa</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/8KmPOPYYGJ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/4AwqQnaHHd</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/6AhuoYYtSD</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/4qCXE8noiQ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/4ft71wlh0D</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/2VocS0zsYG</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/60OUcW8WCY</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/4LGGdVcC3w</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hfCh?c=b&amp;t=p-i657CSw-sPs3l62</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUYR?c=a&amp;t=p-i4vABuk-sJxmTbm</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUdg?c=a&amp;t=p-i6LWBD5-sR1psZs</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hU5a?c=a&amp;t=p-i6Gn16K-s2Du0p2L</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUh1?c=b&amp;t=p-i64ybyV-sPrZX49</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUQb?c=b</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUp1?c=a&amp;t=p-i56HFEE-sPV7YBu</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUs6?c=b&amp;t=p-i3IVVvd-sC7YM7H</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUwm?c=b&amp;t=p-i3uxMq8-sFezCsD</t>
+  </si>
+  <si>
+    <t>https://s.lazada.co.th/s.Z6hUBK?c=a&amp;t=p-i69orjh-sQEG95F</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <sz val="11"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,90 +159,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -427,124 +471,163 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="45" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Product Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Shopee URL</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Lazada URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+    <row r="1" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>ตัวอย่างสินค้า 1</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>ตัวอย่างสินค้า 2</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>ตัวอย่างสินค้า 3</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1"/>
+    <hyperlink ref="C3" r:id="rId2"/>
+    <hyperlink ref="C4" r:id="rId3"/>
+    <hyperlink ref="C5" r:id="rId4"/>
+    <hyperlink ref="C6" r:id="rId5"/>
+    <hyperlink ref="C7" r:id="rId6"/>
+    <hyperlink ref="C8" r:id="rId7"/>
+    <hyperlink ref="C9" r:id="rId8"/>
+    <hyperlink ref="C10" r:id="rId9"/>
+    <hyperlink ref="C11" r:id="rId10"/>
+    <hyperlink ref="D2" r:id="rId11"/>
+    <hyperlink ref="D3" r:id="rId12"/>
+    <hyperlink ref="D4" r:id="rId13"/>
+    <hyperlink ref="D5" r:id="rId14"/>
+    <hyperlink ref="D6" r:id="rId15"/>
+    <hyperlink ref="D7" r:id="rId16"/>
+    <hyperlink ref="D8" r:id="rId17"/>
+    <hyperlink ref="D9" r:id="rId18"/>
+    <hyperlink ref="D10" r:id="rId19"/>
+    <hyperlink ref="D11" r:id="rId20"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update product names, auto-generate hooks for product comments
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -37,9 +37,6 @@
     <t>Shopee Food URL</t>
   </si>
   <si>
-    <t>ตัวอย่างสินค้า 1</t>
-  </si>
-  <si>
     <t>https://s.shopee.co.th/Lk7rJ9Beg</t>
   </si>
   <si>
@@ -52,18 +49,12 @@
     <t>ลด 20% วันนี้เท่านั้น</t>
   </si>
   <si>
-    <t>ตัวอย่างสินค้า 2</t>
-  </si>
-  <si>
     <t>https://s.shopee.co.th/AUqtyHxaLa</t>
   </si>
   <si>
     <t>https://s.lazada.co.th/s.Z6hUYR?c=a&amp;t=p-i4vABuk-sJxmTbm</t>
   </si>
   <si>
-    <t>ตัวอย่างสินค้า 3</t>
-  </si>
-  <si>
     <t>https://s.shopee.co.th/8KmPOPYYGJ</t>
   </si>
   <si>
@@ -154,25 +145,34 @@
     <t>ลองเข้ามาดู Café Amazon (สำนักงานปปง. - SD5580) ที่ Shopee! https://spf.shopee.co.th/40dV0P4yci</t>
   </si>
   <si>
-    <t>ตัวอย่างสินค้า 4</t>
-  </si>
-  <si>
-    <t>ตัวอย่างสินค้า 5</t>
-  </si>
-  <si>
-    <t>ตัวอย่างสินค้า 6</t>
-  </si>
-  <si>
-    <t>ตัวอย่างสินค้า 7</t>
-  </si>
-  <si>
-    <t>ตัวอย่างสินค้า 8</t>
-  </si>
-  <si>
-    <t>ตัวอย่างสินค้า 9</t>
-  </si>
-  <si>
-    <t>ตัวอย่างสินค้า 10</t>
+    <t>Essager หัวชาร์จ GaN 65W ชาร์จเร็ว Type-C/USB-A 2-in-1</t>
+  </si>
+  <si>
+    <t>Biore UV Aqua Rich กันแดดน้ำหนักเบา SPF50+ PA++++ 50g</t>
+  </si>
+  <si>
+    <t>กล่องรองเท้าอะคริลิคใส วางซ้อนกันได้ จัดระเบียบ</t>
+  </si>
+  <si>
+    <t>Baseus Bowie MP1 หูฟัง True Wireless Bluetooth ไร้สาย</t>
+  </si>
+  <si>
+    <t>รองเท้าแมรี่เจน พื้นนุ่ม กันลื่น สไตล์มินิมอล</t>
+  </si>
+  <si>
+    <t>Orsen by Eloop E29 แบตสำรอง 30000mAh QC3.0 PD 45W</t>
+  </si>
+  <si>
+    <t>Gaabor หม้อทอดไร้น้ำมัน 4 ลิตร AF-35M รุ่น Official</t>
+  </si>
+  <si>
+    <t>DHC วิตามินซี Zinc อาหารเสริมบำรุงผิว นำเข้าจากญี่ปุ่น</t>
+  </si>
+  <si>
+    <t>เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ 4 ลิตร ตั้งเวลาผ่านมือถือ</t>
+  </si>
+  <si>
+    <t>Baseus โคมไฟตั้งโต๊ะ LED แม่เหล็กไร้สาย Magnetic</t>
   </si>
 </sst>
 </file>
@@ -234,7 +234,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -242,12 +242,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -260,6 +275,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -594,233 +612,233 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>9</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="D6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
+    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" t="s">
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" t="s">
+    <row r="10" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" t="s">
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G14" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Sony TV and Gold Bar to affiliate products
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,66 @@
       <c r="F20" s="5" t="inlineStr">
         <is>
           <t>ลด 20% วันนี้เท่านั้น</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sony BRAVIA 3 ทีวี 55 นิ้ว รุ่น K-55S30 4K Ultra HD Smart TV (Google TV) | 4K HDR Processor X1™</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/17UzqBrzV</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>สมาร์ททีวี 4K ภาพคมชัด ประกันศูนย์</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>แท่งครึ่งสลึง นน.1.9 กรัม ทองแท้96.5พร้อมใบรับประกันแท่งครึ่งสลึง นน.1.9 กรัม ทองแท้96.5พร้อมใบรับประกัน</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1qZ9BH38am</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ทองคำแท้ 96.5% มีใบรับประกัน ออมทองมั่นใจ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add GQ Underwear, Homkes Hair Dye, and Totori Pillow to affiliate products
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1383,6 +1383,96 @@
       <c r="F22" t="inlineStr">
         <is>
           <t>ทองคำแท้ 96.5% มีใบรับประกัน ออมทองมั่นใจ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>[ลด 50%] GQ Cool Tech กางเกงในไข่เย็น ของแท้ 100% ใส่สบาย ระบายอากาศ ไข่ไม่เหนียวเหนอะหนะ</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/17V045OEX</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>กางเกงในชาย GQ Cool Tech ไข่เย็น สวมสบาย ระบายอากาศได้ดี</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>แชมพูปิดผมขาวหอมเกศ พร้อมบำรุงเส้นผม 990 บาท (แบบขวด 300 มล.)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/70HFL22eBB</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>แชมพูปิดผมขาวหอมเกศ กลิ่นหอม บำรุงเส้นผมดกดำเป็นธรรมชาติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TOTORI หมอน รุ่น คลาวด์(Cloud model) , หมอนหนุน</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7VDVvyHrzL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>หมอนหนุนคุณภาพสูง TOTORI รุ่นคลาวด์ นุ่มสบาย รองรับสรีระได้ดี</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update affiliate products - add ShopeeVIP Xiaomi Watch & Redmi Headphones promotion
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -934,6 +934,36 @@
           <t>ลองเข้ามาดู ขาหมูชานเมือง ข้าวมันไก่ อาหารตามสั่ง ก๋วยเตี๋ยว ที่ Shopee! https://spf.shopee.co.th/AAE8Lxgj6W</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>สมาชิก ShopeeVIP ช้อปสินค้าใหม่ ก่อนใคร 🛒✨
+Xiaomi Watch S5 46mm และ REDMI Headphones Neo พร้อมให้ช้อปแล้ว ! ⌚🎧
+🌟 สมาชิก VIP เริ่มช้อปก่อน : 28 พ.ค. 2569 ตั้งเเต่ 00:00 - 23:59 น.
+👥 ลูกค้าทั่วไป เริ่มช้อป ตั้งเเต่ 29 พ.ค. 2569 เวลา 00:00 น. เป็นต้นไป
+สิทธิพิเศษให้คุณ เข้าถึงรอบ pre-sale ได้ก่อนคนทั่วไป
+สมัครเลย &gt;</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5q5LKroEFe</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://scontent.fbkk5-4.fna.fbcdn.net/v/t39.30808-6/706612549_1357361316520621_597935511996535475_n.jpg?_nc_cat=110&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=KYnBiZnB2KAQ7kNvwGd_0x2&amp;_nc_oc=AdqqVXXlly6Ja0QvmQfSBviMXRfDFaNFYMjAwyMfrH8XOzYkr5JUz3-wTzmMDt1AADnu-BGWnhXvLM4b5WmttcHR&amp;_nc_zt=23&amp;_nc_ht=scontent.fbkk5-4.fna&amp;_nc_gid=XrPN1-_yVEKIUhf0Jdf9DQ&amp;_nc_ss=7b2a8&amp;oh=00_Af6uaN09xQ4x_WeCM7QE7fHFFzswwLBJ7fil4BDS6cwHcg&amp;oe=6A1CF754</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="6" t="inlineStr">

</xml_diff>